<commit_message>
docs(data): dong bo data_manifest.json + data_dictionary.xlsx voi CLI hien tai
data_manifest.json cu thieu entry price_limit_violations dau cli.py da ghi -
chay lai `qshield-data manifest --config configs/base.yaml` de dong bo. Cung
cap nhat data_dictionary.xlsx (da co dong exchange_periods trong report.py
tu truoc nhung file .xlsx tracked chua duoc regenerate).

Khong dong data/metadata/universe_asof_20260803.csv: file do chi duoc
regenerate qua `qshield-data fetch`, lenh nay tai du lieu that tu
yfinance/DNSE/vnstock qua mang - ngoai pham vi nhanh nay, va la quyet dinh
cua data owner.
</commit_message>
<xml_diff>
--- a/data/metadata/data_dictionary.xlsx
+++ b/data/metadata/data_dictionary.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -600,7 +600,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lịch sử chuyển sàn</t>
+          <t>Lịch sử chuyển sàn (văn xuôi)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -612,25 +612,52 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>exchange_periods</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>list[dict]</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Lịch sử chuyển sàn dạng máy đọc được, dùng để resolve biên độ giá theo ngày (quality.price_limits). Mỗi phần tử {exchange, from?, until?}, biên đóng. Phải khớp exchange_current ở period hiện hành.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[{'exchange': 'HNX', 'until': '2020-11-30'}, {'exchange': 'HOSE', 'from': '2020-12-01'}]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>data_source</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Nguồn tải giá chính: yahoo | dnse</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>dnse</t>
         </is>

</xml_diff>

<commit_message>
feat(data): migrate price ingestion to FiinPro
</commit_message>
<xml_diff>
--- a/data/metadata/data_dictionary.xlsx
+++ b/data/metadata/data_dictionary.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>yahoo_symbol</t>
+          <t>company_name</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -492,73 +492,73 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Symbol trên Yahoo Finance</t>
+          <t>Tên doanh nghiệp</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HPG.VN</t>
+          <t>Hoà Phát</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>company_name</t>
+          <t>first_trading_date</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>YYYY-MM-DD</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tên doanh nghiệp</t>
+          <t>Ngày giao dịch đầu tiên (best-effort)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Hoà Phát</t>
+          <t>2007-11-15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>first_trading_date</t>
+          <t>exchange_current</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ngày giao dịch đầu tiên (best-effort)</t>
+          <t>Sàn hiện tại</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2007-11-15</t>
+          <t>HOSE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>exchange_current</t>
+          <t>exchange_history</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -573,24 +573,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sàn hiện tại</t>
+          <t>Lịch sử chuyển sàn (văn xuôi)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HOSE</t>
+          <t>HNX→HOSE 2020</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>exchange_history</t>
+          <t>exchange_periods</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>list[dict]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -600,66 +600,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lịch sử chuyển sàn (văn xuôi)</t>
+          <t>Lịch sử chuyển sàn dạng máy đọc được, dùng để resolve biên độ giá theo ngày (quality.price_limits). Mỗi phần tử {exchange, from?, until?}, biên đóng. Phải khớp exchange_current ở period hiện hành.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HNX→HOSE 2020</t>
+          <t>[{'exchange': 'HNX', 'until': '2020-11-30'}, {'exchange': 'HOSE', 'from': '2020-12-01'}]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>exchange_periods</t>
+          <t>data_source</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>list[dict]</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lịch sử chuyển sàn dạng máy đọc được, dùng để resolve biên độ giá theo ngày (quality.price_limits). Mỗi phần tử {exchange, from?, until?}, biên đóng. Phải khớp exchange_current ở period hiện hành.</t>
+          <t>Nguồn giá: fiinpro</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[{'exchange': 'HNX', 'until': '2020-11-30'}, {'exchange': 'HOSE', 'from': '2020-12-01'}]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>data_source</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>enum</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Nguồn tải giá chính: yahoo | dnse</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>dnse</t>
+          <t>fiinpro</t>
         </is>
       </c>
     </row>
@@ -674,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -776,7 +749,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Giá không điều chỉnh</t>
+          <t>Giá GỐC khớp trên sàn (không điều chỉnh)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -799,7 +772,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Giá đã điều chỉnh cổ tức/chia tách</t>
+          <t>Giá đóng cửa điều chỉnh của FiinPro, neo theo ngày export — chỉ dùng tính return, không dùng làm giá hiện tại</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -853,7 +826,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>close × volume</t>
+          <t>Giá trị khớp lệnh (vendor)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -865,79 +838,125 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>quality_flag</t>
+          <t>volume_negotiated</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>float</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>shares</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OK hoặc bitmask lỗi (pipe-separated: NONPOS_PRICE|NONPOS_CLOSE|NEG_VOLUME|ZERO_VOLUME). Yahoo Finance đôi khi forward-fill giá cho ngày HOSE nghỉ (phantom days, close = close ngày trước, volume = 0). Pipeline cross-check với lịch giao dịch VN-Index (vnstock/VCI — feed thật từ broker VN) và loại các ngày phantom này khỏi prices_adjusted trước khi lưu, nên không còn xuất hiện trong dữ liệu cuối.</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+          <t>Khối lượng thoả thuận</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>source_id</t>
+          <t>turnover_negotiated</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>float</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>VND</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Nguồn dữ liệu</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>YF_PRICES</t>
-        </is>
-      </c>
+          <t>Giá trị thoả thuận</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>quality_flag</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>OK hoặc bitmask lỗi (pipe-separated: NONPOS_PRICE|NONPOS_CLOSE|NEG_VOLUME|ZERO_VOLUME|INVALID_OHLC). Ngày không có trong lịch VN-Index bị loại trước khi lưu.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nguồn dữ liệu</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>FIINPRO_XLSX</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>data_version</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>semver</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Phiên bản data run</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>v1.0.0</t>
         </is>
@@ -1148,7 +1167,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>close × volume</t>
+          <t>Giá trị khớp lệnh (vendor)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -1485,7 +1504,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nguồn (vnstock_VCI_VNINDEX / yahoo_^VNINDEX / custom_composite_ew)</t>
+          <t>Nguồn (vnstock_VCI_VNINDEX / custom_composite_ew)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>

</xml_diff>